<commit_message>
Update TEDPIX report generator and workbook
</commit_message>
<xml_diff>
--- a/output/TEDPIX_Total_Index_5Y.xlsx
+++ b/output/TEDPIX_Total_Index_5Y.xlsx
@@ -232,7 +232,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>TEDPIX — Tehran Stock Exchange Total Index (شاخص کل) — 2022 to 2026</a:t>
+              <a:t>TEDPIX Total Index 2022-2026</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -250,7 +250,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="18000">
+            <a:ln w="25000">
               <a:solidFill>
                 <a:srgbClr val="1F4E79"/>
               </a:solidFill>
@@ -280,15 +280,13 @@
           <idx val="1"/>
           <order val="1"/>
           <tx>
-            <v>First close of each year</v>
+            <strRef>
+              <f>'Daily'!D1</f>
+            </strRef>
           </tx>
           <spPr>
-            <a:ln w="0">
+            <a:ln>
               <a:noFill/>
-              <a:solidFill>
-                <a:srgbClr val="548235"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
@@ -308,7 +306,6 @@
           </marker>
           <dLbls>
             <numFmt formatCode="#,##0"/>
-            <dLblPos val="t"/>
             <showVal val="1"/>
             <showCatName val="0"/>
             <showSerName val="0"/>
@@ -328,15 +325,13 @@
           <idx val="2"/>
           <order val="2"/>
           <tx>
-            <v>Last close of each year</v>
+            <strRef>
+              <f>'Daily'!E1</f>
+            </strRef>
           </tx>
           <spPr>
-            <a:ln w="0">
+            <a:ln>
               <a:noFill/>
-              <a:solidFill>
-                <a:srgbClr val="C00000"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
@@ -356,7 +351,6 @@
           </marker>
           <dLbls>
             <numFmt formatCode="#,##0"/>
-            <dLblPos val="t"/>
             <showVal val="1"/>
             <showCatName val="0"/>
             <showSerName val="0"/>
@@ -380,7 +374,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <axPos val="l"/>
+        <axPos val="b"/>
         <title>
           <tx>
             <rich>
@@ -469,7 +463,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="18000">
+            <a:ln w="25000">
               <a:solidFill>
                 <a:srgbClr val="1F4E79"/>
               </a:solidFill>
@@ -504,7 +498,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="18000">
+            <a:ln w="25000">
               <a:solidFill>
                 <a:srgbClr val="2E86AB"/>
               </a:solidFill>
@@ -539,7 +533,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="18000">
+            <a:ln w="25000">
               <a:solidFill>
                 <a:srgbClr val="BF8F00"/>
               </a:solidFill>
@@ -574,7 +568,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="18000">
+            <a:ln w="25000">
               <a:solidFill>
                 <a:srgbClr val="548235"/>
               </a:solidFill>
@@ -609,7 +603,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="18000">
+            <a:ln w="25000">
               <a:solidFill>
                 <a:srgbClr val="C00000"/>
               </a:solidFill>
@@ -643,7 +637,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <axPos val="l"/>
+        <axPos val="b"/>
         <title>
           <tx>
             <rich>
@@ -710,13 +704,18 @@
       <row>4</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="8640000" cy="4320000"/>
+    <ext cx="7920000" cy="4320000"/>
     <graphicFrame>
       <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
+        <cNvPr id="2" name="Chart 1"/>
+        <cNvGraphicFramePr>
+          <a:graphicFrameLocks noGrp="1"/>
+        </cNvGraphicFramePr>
       </nvGraphicFramePr>
-      <xfrm/>
+      <xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId1"/>
@@ -732,13 +731,18 @@
       <row>34</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="8640000" cy="4320000"/>
+    <ext cx="7920000" cy="4320000"/>
     <graphicFrame>
       <nvGraphicFramePr>
-        <cNvPr id="2" name="Chart 2"/>
-        <cNvGraphicFramePr/>
+        <cNvPr id="3" name="Chart 2"/>
+        <cNvGraphicFramePr>
+          <a:graphicFrameLocks noGrp="1"/>
+        </cNvGraphicFramePr>
       </nvGraphicFramePr>
-      <xfrm/>
+      <xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId2"/>

</xml_diff>